<commit_message>
Ultrasound transceiver in BOM
</commit_message>
<xml_diff>
--- a/8Bit_Binary_BCD_Converter/8Bit_Binary_BCD_Converter.xlsx
+++ b/8Bit_Binary_BCD_Converter/8Bit_Binary_BCD_Converter.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxime\Desktop\Projet Perso\C3I\Measure_Glove\C3I_Measure_Glove\8Bit_Binary_BCD_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDDF4FC3-B247-46B5-8135-02A1F89235C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DFE5A46-0885-440E-B124-8067DF60D84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{91DB6C5E-B195-4882-8085-C6ECB97F7383}"/>
   </bookViews>
   <sheets>
     <sheet name="8Bit_Binary_BCD_Converter" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
   <si>
     <t>Reference</t>
   </si>
@@ -86,13 +99,40 @@
   </si>
   <si>
     <t>SN74AHC1G08DCKR</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C242178.html</t>
+  </si>
+  <si>
+    <t>INGHAi</t>
+  </si>
+  <si>
+    <t>GU1008C-40T &amp; GU1008C-40R</t>
+  </si>
+  <si>
+    <t>LCSC Part Number</t>
+  </si>
+  <si>
+    <t>C242178</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>Website</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,6 +263,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -525,7 +573,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -568,11 +616,13 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -606,6 +656,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -946,126 +997,202 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCA6E4FE-84B4-4E4B-82B8-F98FFB62ED8A}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="81.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
+      <c r="L1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>10</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>0.78600000000000003</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>7.86</v>
       </c>
+      <c r="L2" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>10</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>0.58499999999999996</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>5.85</v>
       </c>
+      <c r="L3" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>21</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>10</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>9.9000000000000005E-2</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>0.99</v>
+      </c>
+      <c r="L4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>1.2193000000000001</v>
+      </c>
+      <c r="J5">
+        <f>H5*I5</f>
+        <v>12.193000000000001</v>
+      </c>
+      <c r="L5" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E5" r:id="rId1" xr:uid="{C6A81CEB-94F3-4E53-A3C1-E422D1A3302E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Conversion + Display Schematic. Missing forced ground on ADC booth
</commit_message>
<xml_diff>
--- a/8Bit_Binary_BCD_Converter/8Bit_Binary_BCD_Converter.xlsx
+++ b/8Bit_Binary_BCD_Converter/8Bit_Binary_BCD_Converter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxime\Desktop\Projet Perso\C3I\Measure_Glove\C3I_Measure_Glove\8Bit_Binary_BCD_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DFE5A46-0885-440E-B124-8067DF60D84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C77C9E-A5C0-4068-AC7D-A1D31252EEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{91DB6C5E-B195-4882-8085-C6ECB97F7383}"/>
   </bookViews>
@@ -1061,7 +1061,7 @@
       <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F2" t="s">
@@ -1096,7 +1096,7 @@
       <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F3" t="s">
@@ -1131,7 +1131,7 @@
       <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
       <c r="F4" t="s">
@@ -1192,6 +1192,9 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E5" r:id="rId1" xr:uid="{C6A81CEB-94F3-4E53-A3C1-E422D1A3302E}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{03413D1C-DC4A-4DAE-AC55-E6820237AEE4}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{AA5E507A-13DC-4524-BD60-EABDCC13CC64}"/>
+    <hyperlink ref="E2" r:id="rId4" xr:uid="{B46EE152-959C-4CAE-A1DB-CAB72B2A0E94}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>